<commit_message>
05-01-26 New Topic - ReorderList
</commit_message>
<xml_diff>
--- a/JavaPrograms/Work Done.xlsx
+++ b/JavaPrograms/Work Done.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="2" activeTab="4"/>
+    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="2" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="DSA plan" sheetId="4" r:id="rId1"/>
@@ -4583,15 +4583,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <i/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>

</xml_diff>

<commit_message>
08-01-26 new topic - stack
</commit_message>
<xml_diff>
--- a/JavaPrograms/Work Done.xlsx
+++ b/JavaPrograms/Work Done.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8280" firstSheet="2" activeTab="4"/>
+    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="DSA plan" sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="383">
   <si>
     <r>
       <rPr>
@@ -3852,6 +3852,47 @@
 If all this made sense reading calmly, you’re good.</t>
   </si>
   <si>
+    <t>Stack</t>
+  </si>
+  <si>
+    <t>Think of a stack of plates.
+You put a plate on top
+You remove the top plate
+You can’t remove the middle plate directly
+So stack =
+👉 Last In, First Out (LIFO)
+Why stacks exist in DSA problems:
+To remember something temporarily
+To undo / go back
+To wait until the right moment
+3️⃣ Stack — Normal explanation (pattern view)
+A stack helps when:
+Current decision depends on future elements
+You need to pause processing and resume later
+Order matters more than values
+Common signals:
+“nearest greater”
+“previous smaller”
+parentheses
+backtracking-like behavior
+If you see “wait until”, think stack.</t>
+  </si>
+  <si>
+    <t>Your car-door analogy (validated)
+Order of opening:
+Driver door
+Behind driver
+Opposite to behind driver
+Opposite to driver
+Now real-life constraint:
+You cannot close door #1 until doors #4, #3, #2 are closed.
+The last opened door must be closed first.
+That is exactly a stack.
+So yes:
+First close opposite to driver → then behind → then opposite → then driver
+That is LIFO in real life.</t>
+  </si>
+  <si>
     <t>Space Complexity</t>
   </si>
   <si>
@@ -4740,15 +4781,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <i/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -5355,7 +5396,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -5454,6 +5495,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
@@ -6159,246 +6203,246 @@
   </cols>
   <sheetData>
     <row r="1" ht="90" customHeight="1" spans="1:6">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="58" t="s">
+      <c r="B1" s="58"/>
+      <c r="C1" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="59"/>
-      <c r="E1" s="60" t="s">
+      <c r="D1" s="60"/>
+      <c r="E1" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="60"/>
+      <c r="F1" s="61"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="62" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="16"/>
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="63"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="16"/>
       <c r="B4" s="16"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="61"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="16"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="64"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="61"/>
+      <c r="F6" s="61"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
-      <c r="C7" s="64"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
+      <c r="C7" s="65"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
-      <c r="C8" s="66"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
+      <c r="C8" s="67"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="62" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="18"/>
-      <c r="C9" s="68" t="s">
+      <c r="C9" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="69"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="60"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="61"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="18"/>
       <c r="B10" s="18"/>
-      <c r="C10" s="70"/>
-      <c r="D10" s="71"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
+      <c r="C10" s="71"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="18"/>
       <c r="B11" s="18"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
+      <c r="C11" s="71"/>
+      <c r="D11" s="72"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="18"/>
       <c r="B12" s="18"/>
-      <c r="C12" s="70"/>
-      <c r="D12" s="71"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
+      <c r="C12" s="71"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="18"/>
       <c r="B13" s="18"/>
-      <c r="C13" s="70"/>
-      <c r="D13" s="71"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="18"/>
       <c r="B14" s="18"/>
-      <c r="C14" s="70"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
+      <c r="C14" s="71"/>
+      <c r="D14" s="72"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:6">
       <c r="A15" s="18"/>
       <c r="B15" s="18"/>
-      <c r="C15" s="72"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="18"/>
       <c r="B16" s="18"/>
-      <c r="C16" s="74" t="s">
+      <c r="C16" s="75" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="75"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="61"/>
+      <c r="F16" s="61"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="18"/>
       <c r="B17" s="18"/>
-      <c r="C17" s="76"/>
-      <c r="D17" s="77"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="78"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="18"/>
       <c r="B18" s="18"/>
-      <c r="C18" s="76"/>
-      <c r="D18" s="77"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="60"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="78"/>
+      <c r="E18" s="61"/>
+      <c r="F18" s="61"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="61" t="s">
+      <c r="A19" s="62" t="s">
         <v>8</v>
       </c>
       <c r="B19" s="16"/>
-      <c r="C19" s="76"/>
-      <c r="D19" s="77"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="60"/>
+      <c r="C19" s="77"/>
+      <c r="D19" s="78"/>
+      <c r="E19" s="61"/>
+      <c r="F19" s="61"/>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="16"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="76"/>
-      <c r="D20" s="77"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
+      <c r="C20" s="77"/>
+      <c r="D20" s="78"/>
+      <c r="E20" s="61"/>
+      <c r="F20" s="61"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="16"/>
       <c r="B21" s="16"/>
-      <c r="C21" s="76"/>
-      <c r="D21" s="77"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
+      <c r="C21" s="77"/>
+      <c r="D21" s="78"/>
+      <c r="E21" s="61"/>
+      <c r="F21" s="61"/>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="16"/>
       <c r="B22" s="16"/>
-      <c r="C22" s="76"/>
-      <c r="D22" s="77"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="78"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="16"/>
       <c r="B23" s="16"/>
-      <c r="C23" s="78"/>
-      <c r="D23" s="79"/>
+      <c r="C23" s="79"/>
+      <c r="D23" s="80"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
-      <c r="C24" s="80" t="s">
+      <c r="C24" s="81" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="81"/>
+      <c r="D24" s="82"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="16"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="82"/>
-      <c r="D25" s="83"/>
+      <c r="C25" s="83"/>
+      <c r="D25" s="84"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="82"/>
-      <c r="D26" s="83"/>
+      <c r="C26" s="83"/>
+      <c r="D26" s="84"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
-      <c r="C27" s="82"/>
-      <c r="D27" s="83"/>
+      <c r="C27" s="83"/>
+      <c r="D27" s="84"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="16"/>
       <c r="B28" s="16"/>
-      <c r="C28" s="84"/>
-      <c r="D28" s="85"/>
+      <c r="C28" s="85"/>
+      <c r="D28" s="86"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="16"/>
@@ -6413,7 +6457,7 @@
       <c r="D30" s="20"/>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="62" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="18"/>
@@ -6469,7 +6513,7 @@
       <c r="D39" s="20"/>
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:4">
-      <c r="A40" s="61" t="s">
+      <c r="A40" s="62" t="s">
         <v>11</v>
       </c>
       <c r="B40" s="18"/>
@@ -6531,7 +6575,7 @@
       <c r="D49" s="20"/>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="61" t="s">
+      <c r="A50" s="62" t="s">
         <v>12</v>
       </c>
       <c r="B50" s="18"/>
@@ -6587,7 +6631,7 @@
       <c r="D58" s="20"/>
     </row>
     <row r="59" spans="1:4">
-      <c r="A59" s="61" t="s">
+      <c r="A59" s="62" t="s">
         <v>13</v>
       </c>
       <c r="B59" s="16"/>
@@ -6643,7 +6687,7 @@
       <c r="D67" s="20"/>
     </row>
     <row r="68" spans="1:4">
-      <c r="A68" s="61" t="s">
+      <c r="A68" s="62" t="s">
         <v>14</v>
       </c>
       <c r="B68" s="16"/>
@@ -6705,7 +6749,7 @@
       <c r="D77" s="20"/>
     </row>
     <row r="78" spans="1:4">
-      <c r="A78" s="61" t="s">
+      <c r="A78" s="62" t="s">
         <v>15</v>
       </c>
       <c r="B78" s="16"/>
@@ -6767,7 +6811,7 @@
       <c r="D87" s="20"/>
     </row>
     <row r="88" spans="1:4">
-      <c r="A88" s="61" t="s">
+      <c r="A88" s="62" t="s">
         <v>16</v>
       </c>
       <c r="B88" s="16"/>
@@ -6823,7 +6867,7 @@
       <c r="D96" s="20"/>
     </row>
     <row r="97" spans="1:4">
-      <c r="A97" s="61" t="s">
+      <c r="A97" s="62" t="s">
         <v>17</v>
       </c>
       <c r="B97" s="18"/>
@@ -6879,7 +6923,7 @@
       <c r="D105" s="20"/>
     </row>
     <row r="106" spans="1:4">
-      <c r="A106" s="61" t="s">
+      <c r="A106" s="62" t="s">
         <v>18</v>
       </c>
       <c r="B106" s="16"/>
@@ -6973,7 +7017,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>100</v>
@@ -6981,24 +7025,24 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="3" ht="100.8" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="4" ht="57.6" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -7033,7 +7077,7 @@
       <c r="D1" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="45" t="s">
         <v>23</v>
       </c>
     </row>
@@ -7041,31 +7085,31 @@
       <c r="A2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="45">
+      <c r="B2" s="46">
         <v>45976</v>
       </c>
-      <c r="C2" s="46">
+      <c r="C2" s="47">
         <v>45983</v>
       </c>
       <c r="D2" s="16">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
+      <c r="E2" s="48"/>
     </row>
     <row r="3" ht="115.2" spans="1:5">
       <c r="A3" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="45">
+      <c r="B3" s="46">
         <v>45976</v>
       </c>
-      <c r="C3" s="46">
+      <c r="C3" s="47">
         <v>45983</v>
       </c>
       <c r="D3" s="16">
         <v>4</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="49" t="s">
         <v>26</v>
       </c>
     </row>
@@ -7073,16 +7117,16 @@
       <c r="A4" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="45">
+      <c r="B4" s="46">
         <v>45976</v>
       </c>
-      <c r="C4" s="46">
+      <c r="C4" s="47">
         <v>45983</v>
       </c>
       <c r="D4" s="16">
         <v>3</v>
       </c>
-      <c r="E4" s="49" t="s">
+      <c r="E4" s="50" t="s">
         <v>28</v>
       </c>
     </row>
@@ -7090,125 +7134,125 @@
       <c r="A5" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="45">
+      <c r="B5" s="46">
         <v>45976</v>
       </c>
-      <c r="C5" s="46">
+      <c r="C5" s="47">
         <v>45983</v>
       </c>
       <c r="D5" s="16">
         <v>2</v>
       </c>
-      <c r="E5" s="50"/>
+      <c r="E5" s="51"/>
     </row>
     <row r="6" ht="115.2" spans="1:5">
       <c r="A6" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="45">
+      <c r="B6" s="46">
         <v>45976</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="47">
         <v>45983</v>
       </c>
       <c r="D6" s="16">
         <v>2</v>
       </c>
-      <c r="E6" s="50"/>
+      <c r="E6" s="51"/>
     </row>
     <row r="7" ht="129.6" spans="1:5">
       <c r="A7" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="45">
+      <c r="B7" s="46">
         <v>45976</v>
       </c>
-      <c r="C7" s="46">
+      <c r="C7" s="47">
         <v>45983</v>
       </c>
       <c r="D7" s="16">
         <v>2</v>
       </c>
-      <c r="E7" s="50"/>
-    </row>
-    <row r="8" s="43" customFormat="1" ht="144" spans="1:5">
-      <c r="A8" s="51" t="s">
+      <c r="E7" s="51"/>
+    </row>
+    <row r="8" s="44" customFormat="1" ht="144" spans="1:5">
+      <c r="A8" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="46">
+      <c r="B8" s="47">
         <v>45976</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="47">
         <v>45983</v>
       </c>
-      <c r="D8" s="52">
+      <c r="D8" s="53">
         <v>2</v>
       </c>
-      <c r="E8" s="53"/>
-    </row>
-    <row r="9" s="43" customFormat="1" ht="158.4" spans="1:5">
-      <c r="A9" s="51" t="s">
+      <c r="E8" s="54"/>
+    </row>
+    <row r="9" s="44" customFormat="1" ht="158.4" spans="1:5">
+      <c r="A9" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="46">
+      <c r="B9" s="47">
         <v>45976</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="47">
         <v>45983</v>
       </c>
-      <c r="D9" s="52">
+      <c r="D9" s="53">
         <v>1</v>
       </c>
-      <c r="E9" s="54"/>
-    </row>
-    <row r="10" s="43" customFormat="1" spans="1:5">
-      <c r="A10" s="52" t="s">
+      <c r="E9" s="55"/>
+    </row>
+    <row r="10" s="44" customFormat="1" spans="1:5">
+      <c r="A10" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="46">
+      <c r="B10" s="47">
         <v>45976</v>
       </c>
-      <c r="C10" s="46">
+      <c r="C10" s="47">
         <v>45983</v>
       </c>
-      <c r="D10" s="52">
+      <c r="D10" s="53">
         <v>1</v>
       </c>
-      <c r="E10" s="55" t="s">
+      <c r="E10" s="56" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" s="43" customFormat="1" spans="1:5">
-      <c r="A11" s="52" t="s">
+    <row r="11" s="44" customFormat="1" spans="1:5">
+      <c r="A11" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="46">
+      <c r="B11" s="47">
         <v>45976</v>
       </c>
-      <c r="C11" s="46">
+      <c r="C11" s="47">
         <v>45983</v>
       </c>
-      <c r="D11" s="52">
+      <c r="D11" s="53">
         <v>1</v>
       </c>
-      <c r="E11" s="55" t="s">
+      <c r="E11" s="56" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" s="43" customFormat="1" spans="1:5">
-      <c r="A12" s="52" t="s">
+    <row r="12" s="44" customFormat="1" spans="1:5">
+      <c r="A12" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="46">
+      <c r="B12" s="47">
         <v>45976</v>
       </c>
-      <c r="C12" s="46">
+      <c r="C12" s="47">
         <v>45983</v>
       </c>
-      <c r="D12" s="52">
+      <c r="D12" s="53">
         <v>1</v>
       </c>
-      <c r="E12" s="55" t="s">
+      <c r="E12" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7216,16 +7260,16 @@
       <c r="A13" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="46">
+      <c r="B13" s="47">
         <v>45977</v>
       </c>
-      <c r="C13" s="46">
+      <c r="C13" s="47">
         <v>45982</v>
       </c>
       <c r="D13" s="16">
         <v>1</v>
       </c>
-      <c r="E13" s="55" t="s">
+      <c r="E13" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7233,16 +7277,16 @@
       <c r="A14" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="46">
+      <c r="B14" s="47">
         <v>45980</v>
       </c>
-      <c r="C14" s="46">
+      <c r="C14" s="47">
         <v>45982</v>
       </c>
       <c r="D14" s="16">
         <v>1</v>
       </c>
-      <c r="E14" s="55" t="s">
+      <c r="E14" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7250,16 +7294,16 @@
       <c r="A15" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="46">
+      <c r="B15" s="47">
         <v>45980</v>
       </c>
-      <c r="C15" s="46">
+      <c r="C15" s="47">
         <v>45982</v>
       </c>
       <c r="D15" s="16">
         <v>1</v>
       </c>
-      <c r="E15" s="55" t="s">
+      <c r="E15" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7267,16 +7311,16 @@
       <c r="A16" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="46">
+      <c r="B16" s="47">
         <v>45980</v>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="47">
         <v>45982</v>
       </c>
       <c r="D16" s="16">
         <v>1</v>
       </c>
-      <c r="E16" s="55" t="s">
+      <c r="E16" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7284,16 +7328,16 @@
       <c r="A17" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="46">
+      <c r="B17" s="47">
         <v>45980</v>
       </c>
-      <c r="C17" s="46">
+      <c r="C17" s="47">
         <v>45982</v>
       </c>
       <c r="D17" s="16">
         <v>1</v>
       </c>
-      <c r="E17" s="55" t="s">
+      <c r="E17" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7301,16 +7345,16 @@
       <c r="A18" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="46">
+      <c r="B18" s="47">
         <v>45981</v>
       </c>
-      <c r="C18" s="46">
+      <c r="C18" s="47">
         <v>45983</v>
       </c>
       <c r="D18" s="16">
         <v>1</v>
       </c>
-      <c r="E18" s="55" t="s">
+      <c r="E18" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7318,16 +7362,16 @@
       <c r="A19" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="46">
+      <c r="B19" s="47">
         <v>45982</v>
       </c>
-      <c r="C19" s="46">
+      <c r="C19" s="47">
         <v>45984</v>
       </c>
       <c r="D19" s="16">
         <v>1</v>
       </c>
-      <c r="E19" s="55" t="s">
+      <c r="E19" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7335,16 +7379,16 @@
       <c r="A20" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="46">
+      <c r="B20" s="47">
         <v>45983</v>
       </c>
-      <c r="C20" s="46">
+      <c r="C20" s="47">
         <v>45985</v>
       </c>
       <c r="D20" s="16">
         <v>1</v>
       </c>
-      <c r="E20" s="55" t="s">
+      <c r="E20" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7352,16 +7396,16 @@
       <c r="A21" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="46">
+      <c r="B21" s="47">
         <v>45986</v>
       </c>
-      <c r="C21" s="46">
+      <c r="C21" s="47">
         <v>45987</v>
       </c>
       <c r="D21" s="16">
         <v>1</v>
       </c>
-      <c r="E21" s="55" t="s">
+      <c r="E21" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7369,16 +7413,16 @@
       <c r="A22" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="46">
+      <c r="B22" s="47">
         <v>45986</v>
       </c>
-      <c r="C22" s="46">
+      <c r="C22" s="47">
         <v>45987</v>
       </c>
       <c r="D22" s="16">
         <v>1</v>
       </c>
-      <c r="E22" s="55" t="s">
+      <c r="E22" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7386,16 +7430,16 @@
       <c r="A23" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="46">
+      <c r="B23" s="47">
         <v>45986</v>
       </c>
-      <c r="C23" s="46">
+      <c r="C23" s="47">
         <v>45987</v>
       </c>
       <c r="D23" s="16">
         <v>1</v>
       </c>
-      <c r="E23" s="55" t="s">
+      <c r="E23" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7403,16 +7447,16 @@
       <c r="A24" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="46">
+      <c r="B24" s="47">
         <v>45986</v>
       </c>
-      <c r="C24" s="46">
+      <c r="C24" s="47">
         <v>45987</v>
       </c>
       <c r="D24" s="16">
         <v>1</v>
       </c>
-      <c r="E24" s="55" t="s">
+      <c r="E24" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7420,16 +7464,16 @@
       <c r="A25" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="46">
+      <c r="B25" s="47">
         <v>45986</v>
       </c>
-      <c r="C25" s="46">
+      <c r="C25" s="47">
         <v>45987</v>
       </c>
       <c r="D25" s="16">
         <v>1</v>
       </c>
-      <c r="E25" s="55" t="s">
+      <c r="E25" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7437,16 +7481,16 @@
       <c r="A26" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="46">
+      <c r="B26" s="47">
         <v>45986</v>
       </c>
-      <c r="C26" s="46">
+      <c r="C26" s="47">
         <v>45987</v>
       </c>
       <c r="D26" s="16">
         <v>1</v>
       </c>
-      <c r="E26" s="55" t="s">
+      <c r="E26" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7454,16 +7498,16 @@
       <c r="A27" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="46">
+      <c r="B27" s="47">
         <v>45986</v>
       </c>
-      <c r="C27" s="46">
+      <c r="C27" s="47">
         <v>45987</v>
       </c>
       <c r="D27" s="16">
         <v>1</v>
       </c>
-      <c r="E27" s="55" t="s">
+      <c r="E27" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7471,16 +7515,16 @@
       <c r="A28" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="46">
+      <c r="B28" s="47">
         <v>45986</v>
       </c>
-      <c r="C28" s="46">
+      <c r="C28" s="47">
         <v>45987</v>
       </c>
       <c r="D28" s="16">
         <v>1</v>
       </c>
-      <c r="E28" s="55" t="s">
+      <c r="E28" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7488,16 +7532,16 @@
       <c r="A29" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="46">
+      <c r="B29" s="47">
         <v>45986</v>
       </c>
-      <c r="C29" s="46">
+      <c r="C29" s="47">
         <v>45987</v>
       </c>
       <c r="D29" s="16">
         <v>1</v>
       </c>
-      <c r="E29" s="55" t="s">
+      <c r="E29" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7505,16 +7549,16 @@
       <c r="A30" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B30" s="46">
+      <c r="B30" s="47">
         <v>45986</v>
       </c>
-      <c r="C30" s="46">
+      <c r="C30" s="47">
         <v>45987</v>
       </c>
       <c r="D30" s="16">
         <v>1</v>
       </c>
-      <c r="E30" s="55" t="s">
+      <c r="E30" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7522,16 +7566,16 @@
       <c r="A31" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="46">
+      <c r="B31" s="47">
         <v>45992</v>
       </c>
-      <c r="C31" s="46">
+      <c r="C31" s="47">
         <v>45993</v>
       </c>
       <c r="D31" s="16">
         <v>1</v>
       </c>
-      <c r="E31" s="55" t="s">
+      <c r="E31" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7539,16 +7583,16 @@
       <c r="A32" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="46">
+      <c r="B32" s="47">
         <v>45992</v>
       </c>
-      <c r="C32" s="46">
+      <c r="C32" s="47">
         <v>45993</v>
       </c>
       <c r="D32" s="16">
         <v>1</v>
       </c>
-      <c r="E32" s="55" t="s">
+      <c r="E32" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7556,16 +7600,16 @@
       <c r="A33" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="46">
+      <c r="B33" s="47">
         <v>45992</v>
       </c>
-      <c r="C33" s="46">
+      <c r="C33" s="47">
         <v>45993</v>
       </c>
       <c r="D33" s="16">
         <v>1</v>
       </c>
-      <c r="E33" s="55" t="s">
+      <c r="E33" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7573,16 +7617,16 @@
       <c r="A34" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="46">
+      <c r="B34" s="47">
         <v>45993</v>
       </c>
-      <c r="C34" s="46">
+      <c r="C34" s="47">
         <v>45993</v>
       </c>
       <c r="D34" s="16">
         <v>1</v>
       </c>
-      <c r="E34" s="55" t="s">
+      <c r="E34" s="56" t="s">
         <v>35</v>
       </c>
     </row>
@@ -8196,21 +8240,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="40" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="40" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="40" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="2" ht="409.5" spans="1:3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="41" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="42" t="s">
         <v>64</v>
       </c>
       <c r="C2" s="23" t="s">
@@ -8323,7 +8367,7 @@
       <c r="A15" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="43" t="s">
         <v>88</v>
       </c>
       <c r="C15" s="20"/>
@@ -8561,7 +8605,7 @@
       <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="34">
+      <c r="A2" s="35">
         <v>45962</v>
       </c>
       <c r="B2" s="20"/>
@@ -8570,7 +8614,7 @@
       <c r="A3" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="36" t="s">
         <v>91</v>
       </c>
     </row>
@@ -8578,7 +8622,7 @@
       <c r="A4" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="36" t="s">
         <v>93</v>
       </c>
     </row>
@@ -8586,21 +8630,21 @@
       <c r="A5" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="36" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="36">
+      <c r="A6" s="37">
         <v>45969</v>
       </c>
       <c r="B6" s="20"/>
     </row>
-    <row r="7" s="33" customFormat="1" ht="57.6" spans="1:2">
-      <c r="A7" s="37" t="s">
+    <row r="7" s="34" customFormat="1" ht="57.6" spans="1:2">
+      <c r="A7" s="38" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="39" t="s">
         <v>97</v>
       </c>
     </row>
@@ -9391,9 +9435,16 @@
         <v>287</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
-      <c r="A86" s="16"/>
-      <c r="B86" s="16"/>
+    <row r="86" ht="302.4" spans="1:3">
+      <c r="A86" s="16" t="s">
+        <v>288</v>
+      </c>
+      <c r="B86" s="18" t="s">
+        <v>289</v>
+      </c>
+      <c r="C86" s="33" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="16"/>
@@ -9466,7 +9517,7 @@
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="16" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11" spans="1:1">
@@ -9504,7 +9555,7 @@
         <v>38</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="18" spans="1:1">
@@ -9514,76 +9565,76 @@
     </row>
     <row r="19" ht="72" spans="1:1">
       <c r="A19" s="2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="20" ht="72" spans="1:1">
       <c r="A20" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="21" ht="100.8" spans="1:2">
       <c r="A21" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="19" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B22" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="23" ht="57.6" spans="1:2">
       <c r="A23" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="24" ht="72" spans="1:2">
       <c r="A24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="25" ht="86.4" spans="1:2">
       <c r="A25" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="26" ht="43.2" spans="1:2">
       <c r="A26" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="27" ht="28.8" spans="1:2">
       <c r="A27" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="28" ht="43.2" spans="1:2">
       <c r="A28" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -9603,27 +9654,27 @@
   <sheetData>
     <row r="2" spans="1:1">
       <c r="A2" s="14" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="8" ht="15" spans="1:1">
       <c r="A8" s="15" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" ht="120" customHeight="1" spans="1:1">
       <c r="A9" s="9" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
   </sheetData>
@@ -9647,201 +9698,201 @@
   <sheetData>
     <row r="1" spans="2:3">
       <c r="B1" s="7" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="2" spans="2:3">
       <c r="B2" s="8" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="8" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="8" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>319</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="8" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="8" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="8" ht="43.2" spans="2:3">
       <c r="B8" s="8" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" spans="2:2">
       <c r="B9" s="10" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="10" spans="2:2">
       <c r="B10" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
     <row r="11" ht="23.4" spans="2:2">
       <c r="B11" s="11" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="12" spans="2:2">
       <c r="B12" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="13" spans="2:2">
       <c r="B13" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="14" spans="2:2">
       <c r="B14" s="12" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="15" spans="2:2">
       <c r="B15" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" spans="2:2">
       <c r="B16" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="17" spans="2:2">
       <c r="B17" s="12" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="18" spans="2:2">
       <c r="B18" s="12" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="19" spans="2:2">
       <c r="B19" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="20" spans="2:2">
       <c r="B20" s="12" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="21" spans="2:2">
       <c r="B21" s="12" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="22" spans="2:2">
       <c r="B22" s="12" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="23" spans="2:2">
       <c r="B23" s="12" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="24" spans="2:2">
       <c r="B24" s="12" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="25" spans="2:2">
       <c r="B25" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="26" ht="23.4" spans="2:2">
       <c r="B26" s="11" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="27" spans="2:2">
       <c r="B27" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="28" spans="2:2">
       <c r="B28" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="29" spans="2:2">
       <c r="B29" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="30" spans="2:2">
       <c r="B30" s="12" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="31" spans="2:2">
       <c r="B31" s="12" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="32" spans="2:2">
       <c r="B32" s="12" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="33" spans="2:2">
       <c r="B33" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="34" spans="2:2">
       <c r="B34" s="12" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
     </row>
     <row r="35" spans="2:2">
       <c r="B35" s="12" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="36" spans="2:2">
@@ -9866,83 +9917,83 @@
     </row>
     <row r="40" spans="2:2">
       <c r="B40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="41" ht="23.4" spans="2:2">
       <c r="B41" s="11" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="42" spans="2:2">
       <c r="B42" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="43" spans="2:2">
       <c r="B43" s="12" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="44" spans="2:2">
       <c r="B44" s="12" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="45" spans="2:2">
       <c r="B45" s="12" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="46" spans="2:2">
       <c r="B46" s="12" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="47" spans="2:2">
       <c r="B47" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="48" spans="2:2">
       <c r="B48" s="13" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="49" spans="2:2">
       <c r="B49" s="13" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="50" spans="2:2">
       <c r="B50" s="13" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="51" spans="2:2">
       <c r="B51" s="13" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="52" spans="2:2">
       <c r="B52" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="54" ht="13" customHeight="1"/>
     <row r="55" ht="22" customHeight="1" spans="2:2">
       <c r="B55" s="11" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="56" spans="2:2">
       <c r="B56" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
     </row>
     <row r="57" spans="2:2">
       <c r="B57" s="12" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="58" spans="2:2">
@@ -9957,17 +10008,17 @@
     </row>
     <row r="60" spans="2:2">
       <c r="B60" s="12" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="61" spans="2:2">
       <c r="B61" s="12" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="62" spans="2:2">
       <c r="B62" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
   </sheetData>
@@ -9984,7 +10035,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -9999,7 +10050,7 @@
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
       <c r="N1" s="5" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="O1" s="6"/>
       <c r="P1" s="6"/>
@@ -10241,7 +10292,7 @@
     </row>
     <row r="12" spans="1:21">
       <c r="A12" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -10427,7 +10478,7 @@
     </row>
     <row r="22" spans="1:21">
       <c r="A22" s="4" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>

</xml_diff>

<commit_message>
11-01-26 new topic - stack Valid Parenthesis practice
</commit_message>
<xml_diff>
--- a/JavaPrograms/Work Done.xlsx
+++ b/JavaPrograms/Work Done.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="385">
   <si>
     <r>
       <rPr>
@@ -3707,6 +3707,7 @@
 [5 | next] → [7 | next] → [9 | null]
 A linked list is just boxes connected by arrows.
 2️⃣ What does a pointer store?
+222
 A pointer stores the address of a box, not the value.
 It’s like:
 not holding the house
@@ -3893,6 +3894,80 @@
 How to explain it more simply (even cleaner)
 Here’s the simplest version you can say without thinking:
 “Whenever things must be closed in the reverse order of opening, we use a stack.”</t>
+  </si>
+  <si>
+    <t>Monotonic Stack</t>
+  </si>
+  <si>
+    <t>Imagine you’re standing in a line of people.
+You want to know:
+“For each person, who is the next taller person in front?”
+You could check everyone one by one (slow).
+Instead, you do this:
+Keep a stack of people who still haven’t found a taller person.
+When a taller person arrives, they become the answer for many behind them.
+That’s monotonic stack.
+2️⃣ What “monotonic” means (simple)
+Monotonic = always in one order
+Two types:
+✅ Monotonic Increasing Stack
+Stack values go like:
+1 3 5 8
+(never decreases)
+✅ Monotonic Decreasing Stack
+Stack values go like:
+8 6 4 2
+(never increases)
+3️⃣ Why do we even need this?
+Because it solves problems like:
+Next Greater Element
+Next Smaller Element
+Previous Greater/Smaller
+Daily Temperatures
+Stock Span
+Largest Rectangle in Histogram
+These problems share one demand:
+“Find the next thing to the right (or left) that breaks a condition.”
+4️⃣ The one rule you must memorize
+Pop until the stack becomes valid again.
+That’s it.
+Monotonic stack is basically:
+✅ keep stack ordered
+✅ when new element breaks order → popImagine you’re standing in a line of people.
+You want to know:
+“For each person, who is the next taller person in front?”
+You could check everyone one by one (slow).
+Instead, you do this:
+Keep a stack of people who still haven’t found a taller person.
+When a taller person arrives, they become the answer for many behind them.
+That’s monotonic stack.
+2️⃣ What “monotonic” means (simple)
+Monotonic = always in one order
+Two types
+✅ Monotonic Increasing Stack
+Stack values go like:
+1 3 5 8
+(never decreases)
+✅ Monotonic Decreasing Stack
+Stack values go like:
+8 6 4 2
+(never increases)
+3️⃣ Why do we even need this?
+Because it solves problems like:
+Next Greater Element
+Next Smaller Element
+Previous Greater/Smaller
+Daily Temperatures
+Stock Span
+Largest Rectangle in Histogram
+These problems share one demand:
+“Find the next thing to the right (or left) that breaks a condition.”
+4️⃣ The one rule you must memorize
+Pop until the stack becomes valid again.
+That’s it.
+Monotonic stack is basically:
+✅ keep stack ordered
+✅ when new element breaks order → pop</t>
   </si>
   <si>
     <t>Space Complexity</t>
@@ -4783,15 +4858,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <i/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -5398,7 +5473,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -5497,9 +5572,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
@@ -6205,246 +6277,246 @@
   </cols>
   <sheetData>
     <row r="1" ht="90" customHeight="1" spans="1:6">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="59" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="60"/>
-      <c r="E1" s="61" t="s">
+      <c r="D1" s="59"/>
+      <c r="E1" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="61"/>
+      <c r="F1" s="60"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="61" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="16"/>
-      <c r="C2" s="63" t="s">
+      <c r="C2" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="64"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="16"/>
       <c r="B4" s="16"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="61"/>
-      <c r="F4" s="61"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="16"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
-      <c r="C7" s="65"/>
-      <c r="D7" s="66"/>
-      <c r="E7" s="61"/>
-      <c r="F7" s="61"/>
+      <c r="C7" s="64"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="60"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
-      <c r="C8" s="67"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
+      <c r="C8" s="66"/>
+      <c r="D8" s="67"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="60"/>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="62" t="s">
+      <c r="A9" s="61" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="18"/>
-      <c r="C9" s="69" t="s">
+      <c r="C9" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="70"/>
-      <c r="E9" s="61"/>
-      <c r="F9" s="61"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="60"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="18"/>
       <c r="B10" s="18"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
+      <c r="C10" s="70"/>
+      <c r="D10" s="71"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="18"/>
       <c r="B11" s="18"/>
-      <c r="C11" s="71"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="61"/>
-      <c r="F11" s="61"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="71"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="18"/>
       <c r="B12" s="18"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="71"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="18"/>
       <c r="B13" s="18"/>
-      <c r="C13" s="71"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="61"/>
-      <c r="F13" s="61"/>
+      <c r="C13" s="70"/>
+      <c r="D13" s="71"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="60"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="18"/>
       <c r="B14" s="18"/>
-      <c r="C14" s="71"/>
-      <c r="D14" s="72"/>
-      <c r="E14" s="61"/>
-      <c r="F14" s="61"/>
+      <c r="C14" s="70"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="60"/>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:6">
       <c r="A15" s="18"/>
       <c r="B15" s="18"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="74"/>
-      <c r="E15" s="61"/>
-      <c r="F15" s="61"/>
+      <c r="C15" s="72"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="60"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="18"/>
       <c r="B16" s="18"/>
-      <c r="C16" s="75" t="s">
+      <c r="C16" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="76"/>
-      <c r="E16" s="61"/>
-      <c r="F16" s="61"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="60"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="18"/>
       <c r="B17" s="18"/>
-      <c r="C17" s="77"/>
-      <c r="D17" s="78"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
+      <c r="C17" s="76"/>
+      <c r="D17" s="77"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="18"/>
       <c r="B18" s="18"/>
-      <c r="C18" s="77"/>
-      <c r="D18" s="78"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="61"/>
+      <c r="C18" s="76"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="60"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="62" t="s">
+      <c r="A19" s="61" t="s">
         <v>8</v>
       </c>
       <c r="B19" s="16"/>
-      <c r="C19" s="77"/>
-      <c r="D19" s="78"/>
-      <c r="E19" s="61"/>
-      <c r="F19" s="61"/>
+      <c r="C19" s="76"/>
+      <c r="D19" s="77"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="60"/>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="16"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="77"/>
-      <c r="D20" s="78"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61"/>
+      <c r="C20" s="76"/>
+      <c r="D20" s="77"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="60"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="16"/>
       <c r="B21" s="16"/>
-      <c r="C21" s="77"/>
-      <c r="D21" s="78"/>
-      <c r="E21" s="61"/>
-      <c r="F21" s="61"/>
+      <c r="C21" s="76"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="60"/>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="16"/>
       <c r="B22" s="16"/>
-      <c r="C22" s="77"/>
-      <c r="D22" s="78"/>
+      <c r="C22" s="76"/>
+      <c r="D22" s="77"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="16"/>
       <c r="B23" s="16"/>
-      <c r="C23" s="79"/>
-      <c r="D23" s="80"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="79"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
-      <c r="C24" s="81" t="s">
+      <c r="C24" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="82"/>
+      <c r="D24" s="81"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="16"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="83"/>
-      <c r="D25" s="84"/>
+      <c r="C25" s="82"/>
+      <c r="D25" s="83"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="83"/>
-      <c r="D26" s="84"/>
+      <c r="C26" s="82"/>
+      <c r="D26" s="83"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
-      <c r="C27" s="83"/>
-      <c r="D27" s="84"/>
+      <c r="C27" s="82"/>
+      <c r="D27" s="83"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="16"/>
       <c r="B28" s="16"/>
-      <c r="C28" s="85"/>
-      <c r="D28" s="86"/>
+      <c r="C28" s="84"/>
+      <c r="D28" s="85"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="16"/>
@@ -6459,7 +6531,7 @@
       <c r="D30" s="20"/>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="62" t="s">
+      <c r="A31" s="61" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="18"/>
@@ -6515,7 +6587,7 @@
       <c r="D39" s="20"/>
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:4">
-      <c r="A40" s="62" t="s">
+      <c r="A40" s="61" t="s">
         <v>11</v>
       </c>
       <c r="B40" s="18"/>
@@ -6577,7 +6649,7 @@
       <c r="D49" s="20"/>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="62" t="s">
+      <c r="A50" s="61" t="s">
         <v>12</v>
       </c>
       <c r="B50" s="18"/>
@@ -6633,7 +6705,7 @@
       <c r="D58" s="20"/>
     </row>
     <row r="59" spans="1:4">
-      <c r="A59" s="62" t="s">
+      <c r="A59" s="61" t="s">
         <v>13</v>
       </c>
       <c r="B59" s="16"/>
@@ -6689,7 +6761,7 @@
       <c r="D67" s="20"/>
     </row>
     <row r="68" spans="1:4">
-      <c r="A68" s="62" t="s">
+      <c r="A68" s="61" t="s">
         <v>14</v>
       </c>
       <c r="B68" s="16"/>
@@ -6751,7 +6823,7 @@
       <c r="D77" s="20"/>
     </row>
     <row r="78" spans="1:4">
-      <c r="A78" s="62" t="s">
+      <c r="A78" s="61" t="s">
         <v>15</v>
       </c>
       <c r="B78" s="16"/>
@@ -6813,7 +6885,7 @@
       <c r="D87" s="20"/>
     </row>
     <row r="88" spans="1:4">
-      <c r="A88" s="62" t="s">
+      <c r="A88" s="61" t="s">
         <v>16</v>
       </c>
       <c r="B88" s="16"/>
@@ -6869,7 +6941,7 @@
       <c r="D96" s="20"/>
     </row>
     <row r="97" spans="1:4">
-      <c r="A97" s="62" t="s">
+      <c r="A97" s="61" t="s">
         <v>17</v>
       </c>
       <c r="B97" s="18"/>
@@ -6925,7 +6997,7 @@
       <c r="D105" s="20"/>
     </row>
     <row r="106" spans="1:4">
-      <c r="A106" s="62" t="s">
+      <c r="A106" s="61" t="s">
         <v>18</v>
       </c>
       <c r="B106" s="16"/>
@@ -7019,7 +7091,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>100</v>
@@ -7027,24 +7099,24 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="3" ht="100.8" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="4" ht="57.6" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -7079,7 +7151,7 @@
       <c r="D1" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="45" t="s">
+      <c r="E1" s="44" t="s">
         <v>23</v>
       </c>
     </row>
@@ -7087,31 +7159,31 @@
       <c r="A2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="46">
+      <c r="B2" s="45">
         <v>45976</v>
       </c>
-      <c r="C2" s="47">
+      <c r="C2" s="46">
         <v>45983</v>
       </c>
       <c r="D2" s="16">
         <v>4</v>
       </c>
-      <c r="E2" s="48"/>
+      <c r="E2" s="47"/>
     </row>
     <row r="3" ht="115.2" spans="1:5">
       <c r="A3" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="46">
+      <c r="B3" s="45">
         <v>45976</v>
       </c>
-      <c r="C3" s="47">
+      <c r="C3" s="46">
         <v>45983</v>
       </c>
       <c r="D3" s="16">
         <v>4</v>
       </c>
-      <c r="E3" s="49" t="s">
+      <c r="E3" s="48" t="s">
         <v>26</v>
       </c>
     </row>
@@ -7119,16 +7191,16 @@
       <c r="A4" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="46">
+      <c r="B4" s="45">
         <v>45976</v>
       </c>
-      <c r="C4" s="47">
+      <c r="C4" s="46">
         <v>45983</v>
       </c>
       <c r="D4" s="16">
         <v>3</v>
       </c>
-      <c r="E4" s="50" t="s">
+      <c r="E4" s="49" t="s">
         <v>28</v>
       </c>
     </row>
@@ -7136,125 +7208,125 @@
       <c r="A5" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="46">
+      <c r="B5" s="45">
         <v>45976</v>
       </c>
-      <c r="C5" s="47">
+      <c r="C5" s="46">
         <v>45983</v>
       </c>
       <c r="D5" s="16">
         <v>2</v>
       </c>
-      <c r="E5" s="51"/>
+      <c r="E5" s="50"/>
     </row>
     <row r="6" ht="115.2" spans="1:5">
       <c r="A6" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="46">
+      <c r="B6" s="45">
         <v>45976</v>
       </c>
-      <c r="C6" s="47">
+      <c r="C6" s="46">
         <v>45983</v>
       </c>
       <c r="D6" s="16">
         <v>2</v>
       </c>
-      <c r="E6" s="51"/>
+      <c r="E6" s="50"/>
     </row>
     <row r="7" ht="129.6" spans="1:5">
       <c r="A7" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="46">
+      <c r="B7" s="45">
         <v>45976</v>
       </c>
-      <c r="C7" s="47">
+      <c r="C7" s="46">
         <v>45983</v>
       </c>
       <c r="D7" s="16">
         <v>2</v>
       </c>
-      <c r="E7" s="51"/>
-    </row>
-    <row r="8" s="44" customFormat="1" ht="144" spans="1:5">
-      <c r="A8" s="52" t="s">
+      <c r="E7" s="50"/>
+    </row>
+    <row r="8" s="43" customFormat="1" ht="144" spans="1:5">
+      <c r="A8" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="47">
+      <c r="B8" s="46">
         <v>45976</v>
       </c>
-      <c r="C8" s="47">
+      <c r="C8" s="46">
         <v>45983</v>
       </c>
-      <c r="D8" s="53">
+      <c r="D8" s="52">
         <v>2</v>
       </c>
-      <c r="E8" s="54"/>
-    </row>
-    <row r="9" s="44" customFormat="1" ht="158.4" spans="1:5">
-      <c r="A9" s="52" t="s">
+      <c r="E8" s="53"/>
+    </row>
+    <row r="9" s="43" customFormat="1" ht="158.4" spans="1:5">
+      <c r="A9" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="47">
+      <c r="B9" s="46">
         <v>45976</v>
       </c>
-      <c r="C9" s="47">
+      <c r="C9" s="46">
         <v>45983</v>
       </c>
-      <c r="D9" s="53">
+      <c r="D9" s="52">
         <v>1</v>
       </c>
-      <c r="E9" s="55"/>
-    </row>
-    <row r="10" s="44" customFormat="1" spans="1:5">
-      <c r="A10" s="53" t="s">
+      <c r="E9" s="54"/>
+    </row>
+    <row r="10" s="43" customFormat="1" spans="1:5">
+      <c r="A10" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="47">
+      <c r="B10" s="46">
         <v>45976</v>
       </c>
-      <c r="C10" s="47">
+      <c r="C10" s="46">
         <v>45983</v>
       </c>
-      <c r="D10" s="53">
+      <c r="D10" s="52">
         <v>1</v>
       </c>
-      <c r="E10" s="56" t="s">
+      <c r="E10" s="55" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" s="44" customFormat="1" spans="1:5">
-      <c r="A11" s="53" t="s">
+    <row r="11" s="43" customFormat="1" spans="1:5">
+      <c r="A11" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="47">
+      <c r="B11" s="46">
         <v>45976</v>
       </c>
-      <c r="C11" s="47">
+      <c r="C11" s="46">
         <v>45983</v>
       </c>
-      <c r="D11" s="53">
+      <c r="D11" s="52">
         <v>1</v>
       </c>
-      <c r="E11" s="56" t="s">
+      <c r="E11" s="55" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" s="44" customFormat="1" spans="1:5">
-      <c r="A12" s="53" t="s">
+    <row r="12" s="43" customFormat="1" spans="1:5">
+      <c r="A12" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="47">
+      <c r="B12" s="46">
         <v>45976</v>
       </c>
-      <c r="C12" s="47">
+      <c r="C12" s="46">
         <v>45983</v>
       </c>
-      <c r="D12" s="53">
+      <c r="D12" s="52">
         <v>1</v>
       </c>
-      <c r="E12" s="56" t="s">
+      <c r="E12" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7262,16 +7334,16 @@
       <c r="A13" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="47">
+      <c r="B13" s="46">
         <v>45977</v>
       </c>
-      <c r="C13" s="47">
+      <c r="C13" s="46">
         <v>45982</v>
       </c>
       <c r="D13" s="16">
         <v>1</v>
       </c>
-      <c r="E13" s="56" t="s">
+      <c r="E13" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7279,16 +7351,16 @@
       <c r="A14" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="47">
+      <c r="B14" s="46">
         <v>45980</v>
       </c>
-      <c r="C14" s="47">
+      <c r="C14" s="46">
         <v>45982</v>
       </c>
       <c r="D14" s="16">
         <v>1</v>
       </c>
-      <c r="E14" s="56" t="s">
+      <c r="E14" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7296,16 +7368,16 @@
       <c r="A15" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="47">
+      <c r="B15" s="46">
         <v>45980</v>
       </c>
-      <c r="C15" s="47">
+      <c r="C15" s="46">
         <v>45982</v>
       </c>
       <c r="D15" s="16">
         <v>1</v>
       </c>
-      <c r="E15" s="56" t="s">
+      <c r="E15" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7313,16 +7385,16 @@
       <c r="A16" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="47">
+      <c r="B16" s="46">
         <v>45980</v>
       </c>
-      <c r="C16" s="47">
+      <c r="C16" s="46">
         <v>45982</v>
       </c>
       <c r="D16" s="16">
         <v>1</v>
       </c>
-      <c r="E16" s="56" t="s">
+      <c r="E16" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7330,16 +7402,16 @@
       <c r="A17" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="47">
+      <c r="B17" s="46">
         <v>45980</v>
       </c>
-      <c r="C17" s="47">
+      <c r="C17" s="46">
         <v>45982</v>
       </c>
       <c r="D17" s="16">
         <v>1</v>
       </c>
-      <c r="E17" s="56" t="s">
+      <c r="E17" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7347,16 +7419,16 @@
       <c r="A18" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="47">
+      <c r="B18" s="46">
         <v>45981</v>
       </c>
-      <c r="C18" s="47">
+      <c r="C18" s="46">
         <v>45983</v>
       </c>
       <c r="D18" s="16">
         <v>1</v>
       </c>
-      <c r="E18" s="56" t="s">
+      <c r="E18" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7364,16 +7436,16 @@
       <c r="A19" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="47">
+      <c r="B19" s="46">
         <v>45982</v>
       </c>
-      <c r="C19" s="47">
+      <c r="C19" s="46">
         <v>45984</v>
       </c>
       <c r="D19" s="16">
         <v>1</v>
       </c>
-      <c r="E19" s="56" t="s">
+      <c r="E19" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7381,16 +7453,16 @@
       <c r="A20" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="47">
+      <c r="B20" s="46">
         <v>45983</v>
       </c>
-      <c r="C20" s="47">
+      <c r="C20" s="46">
         <v>45985</v>
       </c>
       <c r="D20" s="16">
         <v>1</v>
       </c>
-      <c r="E20" s="56" t="s">
+      <c r="E20" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7398,16 +7470,16 @@
       <c r="A21" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="47">
+      <c r="B21" s="46">
         <v>45986</v>
       </c>
-      <c r="C21" s="47">
+      <c r="C21" s="46">
         <v>45987</v>
       </c>
       <c r="D21" s="16">
         <v>1</v>
       </c>
-      <c r="E21" s="56" t="s">
+      <c r="E21" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7415,16 +7487,16 @@
       <c r="A22" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="47">
+      <c r="B22" s="46">
         <v>45986</v>
       </c>
-      <c r="C22" s="47">
+      <c r="C22" s="46">
         <v>45987</v>
       </c>
       <c r="D22" s="16">
         <v>1</v>
       </c>
-      <c r="E22" s="56" t="s">
+      <c r="E22" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7432,16 +7504,16 @@
       <c r="A23" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="47">
+      <c r="B23" s="46">
         <v>45986</v>
       </c>
-      <c r="C23" s="47">
+      <c r="C23" s="46">
         <v>45987</v>
       </c>
       <c r="D23" s="16">
         <v>1</v>
       </c>
-      <c r="E23" s="56" t="s">
+      <c r="E23" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7449,16 +7521,16 @@
       <c r="A24" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="47">
+      <c r="B24" s="46">
         <v>45986</v>
       </c>
-      <c r="C24" s="47">
+      <c r="C24" s="46">
         <v>45987</v>
       </c>
       <c r="D24" s="16">
         <v>1</v>
       </c>
-      <c r="E24" s="56" t="s">
+      <c r="E24" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7466,16 +7538,16 @@
       <c r="A25" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="47">
+      <c r="B25" s="46">
         <v>45986</v>
       </c>
-      <c r="C25" s="47">
+      <c r="C25" s="46">
         <v>45987</v>
       </c>
       <c r="D25" s="16">
         <v>1</v>
       </c>
-      <c r="E25" s="56" t="s">
+      <c r="E25" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7483,16 +7555,16 @@
       <c r="A26" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="47">
+      <c r="B26" s="46">
         <v>45986</v>
       </c>
-      <c r="C26" s="47">
+      <c r="C26" s="46">
         <v>45987</v>
       </c>
       <c r="D26" s="16">
         <v>1</v>
       </c>
-      <c r="E26" s="56" t="s">
+      <c r="E26" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7500,16 +7572,16 @@
       <c r="A27" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="47">
+      <c r="B27" s="46">
         <v>45986</v>
       </c>
-      <c r="C27" s="47">
+      <c r="C27" s="46">
         <v>45987</v>
       </c>
       <c r="D27" s="16">
         <v>1</v>
       </c>
-      <c r="E27" s="56" t="s">
+      <c r="E27" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7517,16 +7589,16 @@
       <c r="A28" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="47">
+      <c r="B28" s="46">
         <v>45986</v>
       </c>
-      <c r="C28" s="47">
+      <c r="C28" s="46">
         <v>45987</v>
       </c>
       <c r="D28" s="16">
         <v>1</v>
       </c>
-      <c r="E28" s="56" t="s">
+      <c r="E28" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7534,16 +7606,16 @@
       <c r="A29" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="47">
+      <c r="B29" s="46">
         <v>45986</v>
       </c>
-      <c r="C29" s="47">
+      <c r="C29" s="46">
         <v>45987</v>
       </c>
       <c r="D29" s="16">
         <v>1</v>
       </c>
-      <c r="E29" s="56" t="s">
+      <c r="E29" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7551,16 +7623,16 @@
       <c r="A30" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B30" s="47">
+      <c r="B30" s="46">
         <v>45986</v>
       </c>
-      <c r="C30" s="47">
+      <c r="C30" s="46">
         <v>45987</v>
       </c>
       <c r="D30" s="16">
         <v>1</v>
       </c>
-      <c r="E30" s="56" t="s">
+      <c r="E30" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7568,16 +7640,16 @@
       <c r="A31" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="47">
+      <c r="B31" s="46">
         <v>45992</v>
       </c>
-      <c r="C31" s="47">
+      <c r="C31" s="46">
         <v>45993</v>
       </c>
       <c r="D31" s="16">
         <v>1</v>
       </c>
-      <c r="E31" s="56" t="s">
+      <c r="E31" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7585,16 +7657,16 @@
       <c r="A32" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="47">
+      <c r="B32" s="46">
         <v>45992</v>
       </c>
-      <c r="C32" s="47">
+      <c r="C32" s="46">
         <v>45993</v>
       </c>
       <c r="D32" s="16">
         <v>1</v>
       </c>
-      <c r="E32" s="56" t="s">
+      <c r="E32" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7602,16 +7674,16 @@
       <c r="A33" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="47">
+      <c r="B33" s="46">
         <v>45992</v>
       </c>
-      <c r="C33" s="47">
+      <c r="C33" s="46">
         <v>45993</v>
       </c>
       <c r="D33" s="16">
         <v>1</v>
       </c>
-      <c r="E33" s="56" t="s">
+      <c r="E33" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7619,16 +7691,16 @@
       <c r="A34" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="47">
+      <c r="B34" s="46">
         <v>45993</v>
       </c>
-      <c r="C34" s="47">
+      <c r="C34" s="46">
         <v>45993</v>
       </c>
       <c r="D34" s="16">
         <v>1</v>
       </c>
-      <c r="E34" s="56" t="s">
+      <c r="E34" s="55" t="s">
         <v>35</v>
       </c>
     </row>
@@ -8242,21 +8314,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="2" ht="409.5" spans="1:3">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="40" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="41" t="s">
         <v>64</v>
       </c>
       <c r="C2" s="23" t="s">
@@ -8369,7 +8441,7 @@
       <c r="A15" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="43" t="s">
+      <c r="B15" s="42" t="s">
         <v>88</v>
       </c>
       <c r="C15" s="20"/>
@@ -8607,7 +8679,7 @@
       <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="35">
+      <c r="A2" s="34">
         <v>45962</v>
       </c>
       <c r="B2" s="20"/>
@@ -8616,7 +8688,7 @@
       <c r="A3" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="35" t="s">
         <v>91</v>
       </c>
     </row>
@@ -8624,7 +8696,7 @@
       <c r="A4" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="35" t="s">
         <v>93</v>
       </c>
     </row>
@@ -8632,21 +8704,21 @@
       <c r="A5" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="35" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="37">
+      <c r="A6" s="36">
         <v>45969</v>
       </c>
       <c r="B6" s="20"/>
     </row>
-    <row r="7" s="34" customFormat="1" ht="57.6" spans="1:2">
-      <c r="A7" s="38" t="s">
+    <row r="7" s="33" customFormat="1" ht="57.6" spans="1:2">
+      <c r="A7" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="38" t="s">
         <v>97</v>
       </c>
     </row>
@@ -9444,13 +9516,17 @@
       <c r="B86" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="C86" s="33" t="s">
+      <c r="C86" s="23" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="87" spans="1:2">
-      <c r="A87" s="16"/>
-      <c r="B87" s="16"/>
+    <row r="87" ht="409.5" spans="1:2">
+      <c r="A87" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="B87" s="18" t="s">
+        <v>292</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -9519,7 +9595,7 @@
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="16" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="11" spans="1:1">
@@ -9557,7 +9633,7 @@
         <v>38</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="18" spans="1:1">
@@ -9567,76 +9643,76 @@
     </row>
     <row r="19" ht="72" spans="1:1">
       <c r="A19" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="20" ht="72" spans="1:1">
       <c r="A20" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="21" ht="100.8" spans="1:2">
       <c r="A21" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="19" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B22" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="23" ht="57.6" spans="1:2">
       <c r="A23" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="24" ht="72" spans="1:2">
       <c r="A24" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="25" ht="86.4" spans="1:2">
       <c r="A25" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="26" ht="43.2" spans="1:2">
       <c r="A26" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="27" ht="28.8" spans="1:2">
       <c r="A27" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="28" ht="43.2" spans="1:2">
       <c r="A28" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>
@@ -9656,27 +9732,27 @@
   <sheetData>
     <row r="2" spans="1:1">
       <c r="A2" s="14" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" ht="15" spans="1:1">
       <c r="A8" s="15" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9" ht="120" customHeight="1" spans="1:1">
       <c r="A9" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -9700,201 +9776,201 @@
   <sheetData>
     <row r="1" spans="2:3">
       <c r="B1" s="7" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" spans="2:3">
       <c r="B2" s="8" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="8" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>321</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="8" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="8" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="8" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" ht="43.2" spans="2:3">
       <c r="B8" s="8" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9" spans="2:2">
       <c r="B9" s="10" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10" spans="2:2">
       <c r="B10" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" ht="23.4" spans="2:2">
       <c r="B11" s="11" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" spans="2:2">
       <c r="B12" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="13" spans="2:2">
       <c r="B13" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="14" spans="2:2">
       <c r="B14" s="12" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="2:2">
       <c r="B15" s="12" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="16" spans="2:2">
       <c r="B16" s="12" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" spans="2:2">
       <c r="B17" s="12" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="18" spans="2:2">
       <c r="B18" s="12" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="19" spans="2:2">
       <c r="B19" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="20" spans="2:2">
       <c r="B20" s="12" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="21" spans="2:2">
       <c r="B21" s="12" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="22" spans="2:2">
       <c r="B22" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="23" spans="2:2">
       <c r="B23" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="24" spans="2:2">
       <c r="B24" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="25" spans="2:2">
       <c r="B25" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="26" ht="23.4" spans="2:2">
       <c r="B26" s="11" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="27" spans="2:2">
       <c r="B27" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="28" spans="2:2">
       <c r="B28" s="12" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="29" spans="2:2">
       <c r="B29" s="12" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="30" spans="2:2">
       <c r="B30" s="12" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="31" spans="2:2">
       <c r="B31" s="12" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="32" spans="2:2">
       <c r="B32" s="12" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="33" spans="2:2">
       <c r="B33" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="34" spans="2:2">
       <c r="B34" s="12" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="35" spans="2:2">
       <c r="B35" s="12" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="36" spans="2:2">
@@ -9919,83 +9995,83 @@
     </row>
     <row r="40" spans="2:2">
       <c r="B40" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="41" ht="23.4" spans="2:2">
       <c r="B41" s="11" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="42" spans="2:2">
       <c r="B42" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="43" spans="2:2">
       <c r="B43" s="12" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="44" spans="2:2">
       <c r="B44" s="12" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="45" spans="2:2">
       <c r="B45" s="12" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="46" spans="2:2">
       <c r="B46" s="12" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="47" spans="2:2">
       <c r="B47" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="48" spans="2:2">
       <c r="B48" s="13" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="49" spans="2:2">
       <c r="B49" s="13" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="50" spans="2:2">
       <c r="B50" s="13" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="51" spans="2:2">
       <c r="B51" s="13" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="52" spans="2:2">
       <c r="B52" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="54" ht="13" customHeight="1"/>
     <row r="55" ht="22" customHeight="1" spans="2:2">
       <c r="B55" s="11" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="56" spans="2:2">
       <c r="B56" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="57" spans="2:2">
       <c r="B57" s="12" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="58" spans="2:2">
@@ -10010,17 +10086,17 @@
     </row>
     <row r="60" spans="2:2">
       <c r="B60" s="12" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="61" spans="2:2">
       <c r="B61" s="12" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="62" spans="2:2">
       <c r="B62" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -10037,7 +10113,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" s="3" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -10052,7 +10128,7 @@
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
       <c r="N1" s="5" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="O1" s="6"/>
       <c r="P1" s="6"/>
@@ -10294,7 +10370,7 @@
     </row>
     <row r="12" spans="1:21">
       <c r="A12" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -10480,7 +10556,7 @@
     </row>
     <row r="22" spans="1:21">
       <c r="A22" s="4" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>

</xml_diff>

<commit_message>
16-01-26 Hashing and Sets
</commit_message>
<xml_diff>
--- a/JavaPrograms/Work Done.xlsx
+++ b/JavaPrograms/Work Done.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="2" activeTab="4"/>
+    <workbookView windowWidth="23040" windowHeight="8280" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="DSA plan" sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="387">
   <si>
     <r>
       <rPr>
@@ -3968,6 +3968,24 @@
 Monotonic stack is basically:
 ✅ keep stack ordered
 ✅ when new element breaks order → pop</t>
+  </si>
+  <si>
+    <t>HASHING &amp; SETS</t>
+  </si>
+  <si>
+    <t>This phase is about one superpower:
+O(1) lookup to detect patterns fast
+Hashing solves:
+counting
+uniqueness
+grouping
+existence checking
+ ELI5
+A HashMap is like a notebook:
+you write: “I have seen this before”
+or: “I have seen it 5 times”
+or: “this item belongs to this group”
+Instead of searching full list again and again, you just look in notebook.</t>
   </si>
   <si>
     <t>Space Complexity</t>
@@ -5473,7 +5491,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -5572,6 +5590,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
@@ -6277,246 +6301,246 @@
   </cols>
   <sheetData>
     <row r="1" ht="90" customHeight="1" spans="1:6">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="58" t="s">
+      <c r="B1" s="59"/>
+      <c r="C1" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="59"/>
-      <c r="E1" s="60" t="s">
+      <c r="D1" s="61"/>
+      <c r="E1" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="60"/>
+      <c r="F1" s="62"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="63" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="16"/>
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="63"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="16"/>
       <c r="B4" s="16"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="16"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="64"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
-      <c r="C7" s="64"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
-      <c r="C8" s="66"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="69"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="63" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="18"/>
-      <c r="C9" s="68" t="s">
+      <c r="C9" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="69"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="60"/>
+      <c r="D9" s="71"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="18"/>
       <c r="B10" s="18"/>
-      <c r="C10" s="70"/>
-      <c r="D10" s="71"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
+      <c r="C10" s="72"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="18"/>
       <c r="B11" s="18"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
+      <c r="C11" s="72"/>
+      <c r="D11" s="73"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="62"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="18"/>
       <c r="B12" s="18"/>
-      <c r="C12" s="70"/>
-      <c r="D12" s="71"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="73"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="18"/>
       <c r="B13" s="18"/>
-      <c r="C13" s="70"/>
-      <c r="D13" s="71"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="62"/>
+      <c r="F13" s="62"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="18"/>
       <c r="B14" s="18"/>
-      <c r="C14" s="70"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
+      <c r="C14" s="72"/>
+      <c r="D14" s="73"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:6">
       <c r="A15" s="18"/>
       <c r="B15" s="18"/>
-      <c r="C15" s="72"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="62"/>
+      <c r="F15" s="62"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="18"/>
       <c r="B16" s="18"/>
-      <c r="C16" s="74" t="s">
+      <c r="C16" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="75"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="18"/>
       <c r="B17" s="18"/>
-      <c r="C17" s="76"/>
-      <c r="D17" s="77"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
+      <c r="C17" s="78"/>
+      <c r="D17" s="79"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="62"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="18"/>
       <c r="B18" s="18"/>
-      <c r="C18" s="76"/>
-      <c r="D18" s="77"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="60"/>
+      <c r="C18" s="78"/>
+      <c r="D18" s="79"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="61" t="s">
+      <c r="A19" s="63" t="s">
         <v>8</v>
       </c>
       <c r="B19" s="16"/>
-      <c r="C19" s="76"/>
-      <c r="D19" s="77"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="60"/>
+      <c r="C19" s="78"/>
+      <c r="D19" s="79"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="16"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="76"/>
-      <c r="D20" s="77"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
+      <c r="C20" s="78"/>
+      <c r="D20" s="79"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="16"/>
       <c r="B21" s="16"/>
-      <c r="C21" s="76"/>
-      <c r="D21" s="77"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
+      <c r="C21" s="78"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="62"/>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="16"/>
       <c r="B22" s="16"/>
-      <c r="C22" s="76"/>
-      <c r="D22" s="77"/>
+      <c r="C22" s="78"/>
+      <c r="D22" s="79"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="16"/>
       <c r="B23" s="16"/>
-      <c r="C23" s="78"/>
-      <c r="D23" s="79"/>
+      <c r="C23" s="80"/>
+      <c r="D23" s="81"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
-      <c r="C24" s="80" t="s">
+      <c r="C24" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="81"/>
+      <c r="D24" s="83"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="16"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="82"/>
-      <c r="D25" s="83"/>
+      <c r="C25" s="84"/>
+      <c r="D25" s="85"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="82"/>
-      <c r="D26" s="83"/>
+      <c r="C26" s="84"/>
+      <c r="D26" s="85"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
-      <c r="C27" s="82"/>
-      <c r="D27" s="83"/>
+      <c r="C27" s="84"/>
+      <c r="D27" s="85"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="16"/>
       <c r="B28" s="16"/>
-      <c r="C28" s="84"/>
-      <c r="D28" s="85"/>
+      <c r="C28" s="86"/>
+      <c r="D28" s="87"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="16"/>
@@ -6531,7 +6555,7 @@
       <c r="D30" s="20"/>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="63" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="18"/>
@@ -6587,7 +6611,7 @@
       <c r="D39" s="20"/>
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:4">
-      <c r="A40" s="61" t="s">
+      <c r="A40" s="63" t="s">
         <v>11</v>
       </c>
       <c r="B40" s="18"/>
@@ -6649,7 +6673,7 @@
       <c r="D49" s="20"/>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="61" t="s">
+      <c r="A50" s="63" t="s">
         <v>12</v>
       </c>
       <c r="B50" s="18"/>
@@ -6705,7 +6729,7 @@
       <c r="D58" s="20"/>
     </row>
     <row r="59" spans="1:4">
-      <c r="A59" s="61" t="s">
+      <c r="A59" s="63" t="s">
         <v>13</v>
       </c>
       <c r="B59" s="16"/>
@@ -6761,7 +6785,7 @@
       <c r="D67" s="20"/>
     </row>
     <row r="68" spans="1:4">
-      <c r="A68" s="61" t="s">
+      <c r="A68" s="63" t="s">
         <v>14</v>
       </c>
       <c r="B68" s="16"/>
@@ -6823,7 +6847,7 @@
       <c r="D77" s="20"/>
     </row>
     <row r="78" spans="1:4">
-      <c r="A78" s="61" t="s">
+      <c r="A78" s="63" t="s">
         <v>15</v>
       </c>
       <c r="B78" s="16"/>
@@ -6885,7 +6909,7 @@
       <c r="D87" s="20"/>
     </row>
     <row r="88" spans="1:4">
-      <c r="A88" s="61" t="s">
+      <c r="A88" s="63" t="s">
         <v>16</v>
       </c>
       <c r="B88" s="16"/>
@@ -6941,7 +6965,7 @@
       <c r="D96" s="20"/>
     </row>
     <row r="97" spans="1:4">
-      <c r="A97" s="61" t="s">
+      <c r="A97" s="63" t="s">
         <v>17</v>
       </c>
       <c r="B97" s="18"/>
@@ -6997,7 +7021,7 @@
       <c r="D105" s="20"/>
     </row>
     <row r="106" spans="1:4">
-      <c r="A106" s="61" t="s">
+      <c r="A106" s="63" t="s">
         <v>18</v>
       </c>
       <c r="B106" s="16"/>
@@ -7091,7 +7115,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>100</v>
@@ -7099,24 +7123,24 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="3" ht="100.8" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="4" ht="57.6" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>
@@ -7151,7 +7175,7 @@
       <c r="D1" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="46" t="s">
         <v>23</v>
       </c>
     </row>
@@ -7159,31 +7183,31 @@
       <c r="A2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="45">
+      <c r="B2" s="47">
         <v>45976</v>
       </c>
-      <c r="C2" s="46">
+      <c r="C2" s="48">
         <v>45983</v>
       </c>
       <c r="D2" s="16">
         <v>4</v>
       </c>
-      <c r="E2" s="47"/>
+      <c r="E2" s="49"/>
     </row>
     <row r="3" ht="115.2" spans="1:5">
       <c r="A3" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="45">
+      <c r="B3" s="47">
         <v>45976</v>
       </c>
-      <c r="C3" s="46">
+      <c r="C3" s="48">
         <v>45983</v>
       </c>
       <c r="D3" s="16">
         <v>4</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="50" t="s">
         <v>26</v>
       </c>
     </row>
@@ -7191,16 +7215,16 @@
       <c r="A4" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="45">
+      <c r="B4" s="47">
         <v>45976</v>
       </c>
-      <c r="C4" s="46">
+      <c r="C4" s="48">
         <v>45983</v>
       </c>
       <c r="D4" s="16">
         <v>3</v>
       </c>
-      <c r="E4" s="49" t="s">
+      <c r="E4" s="51" t="s">
         <v>28</v>
       </c>
     </row>
@@ -7208,125 +7232,125 @@
       <c r="A5" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="45">
+      <c r="B5" s="47">
         <v>45976</v>
       </c>
-      <c r="C5" s="46">
+      <c r="C5" s="48">
         <v>45983</v>
       </c>
       <c r="D5" s="16">
         <v>2</v>
       </c>
-      <c r="E5" s="50"/>
+      <c r="E5" s="52"/>
     </row>
     <row r="6" ht="115.2" spans="1:5">
       <c r="A6" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="45">
+      <c r="B6" s="47">
         <v>45976</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="48">
         <v>45983</v>
       </c>
       <c r="D6" s="16">
         <v>2</v>
       </c>
-      <c r="E6" s="50"/>
+      <c r="E6" s="52"/>
     </row>
     <row r="7" ht="129.6" spans="1:5">
       <c r="A7" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="45">
+      <c r="B7" s="47">
         <v>45976</v>
       </c>
-      <c r="C7" s="46">
+      <c r="C7" s="48">
         <v>45983</v>
       </c>
       <c r="D7" s="16">
         <v>2</v>
       </c>
-      <c r="E7" s="50"/>
-    </row>
-    <row r="8" s="43" customFormat="1" ht="144" spans="1:5">
-      <c r="A8" s="51" t="s">
+      <c r="E7" s="52"/>
+    </row>
+    <row r="8" s="45" customFormat="1" ht="144" spans="1:5">
+      <c r="A8" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="46">
+      <c r="B8" s="48">
         <v>45976</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="48">
         <v>45983</v>
       </c>
-      <c r="D8" s="52">
+      <c r="D8" s="54">
         <v>2</v>
       </c>
-      <c r="E8" s="53"/>
-    </row>
-    <row r="9" s="43" customFormat="1" ht="158.4" spans="1:5">
-      <c r="A9" s="51" t="s">
+      <c r="E8" s="55"/>
+    </row>
+    <row r="9" s="45" customFormat="1" ht="158.4" spans="1:5">
+      <c r="A9" s="53" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="46">
+      <c r="B9" s="48">
         <v>45976</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="48">
         <v>45983</v>
       </c>
-      <c r="D9" s="52">
+      <c r="D9" s="54">
         <v>1</v>
       </c>
-      <c r="E9" s="54"/>
-    </row>
-    <row r="10" s="43" customFormat="1" spans="1:5">
-      <c r="A10" s="52" t="s">
+      <c r="E9" s="56"/>
+    </row>
+    <row r="10" s="45" customFormat="1" spans="1:5">
+      <c r="A10" s="54" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="46">
+      <c r="B10" s="48">
         <v>45976</v>
       </c>
-      <c r="C10" s="46">
+      <c r="C10" s="48">
         <v>45983</v>
       </c>
-      <c r="D10" s="52">
+      <c r="D10" s="54">
         <v>1</v>
       </c>
-      <c r="E10" s="55" t="s">
+      <c r="E10" s="57" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" s="43" customFormat="1" spans="1:5">
-      <c r="A11" s="52" t="s">
+    <row r="11" s="45" customFormat="1" spans="1:5">
+      <c r="A11" s="54" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="46">
+      <c r="B11" s="48">
         <v>45976</v>
       </c>
-      <c r="C11" s="46">
+      <c r="C11" s="48">
         <v>45983</v>
       </c>
-      <c r="D11" s="52">
+      <c r="D11" s="54">
         <v>1</v>
       </c>
-      <c r="E11" s="55" t="s">
+      <c r="E11" s="57" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" s="43" customFormat="1" spans="1:5">
-      <c r="A12" s="52" t="s">
+    <row r="12" s="45" customFormat="1" spans="1:5">
+      <c r="A12" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="46">
+      <c r="B12" s="48">
         <v>45976</v>
       </c>
-      <c r="C12" s="46">
+      <c r="C12" s="48">
         <v>45983</v>
       </c>
-      <c r="D12" s="52">
+      <c r="D12" s="54">
         <v>1</v>
       </c>
-      <c r="E12" s="55" t="s">
+      <c r="E12" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7334,16 +7358,16 @@
       <c r="A13" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="46">
+      <c r="B13" s="48">
         <v>45977</v>
       </c>
-      <c r="C13" s="46">
+      <c r="C13" s="48">
         <v>45982</v>
       </c>
       <c r="D13" s="16">
         <v>1</v>
       </c>
-      <c r="E13" s="55" t="s">
+      <c r="E13" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7351,16 +7375,16 @@
       <c r="A14" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="46">
+      <c r="B14" s="48">
         <v>45980</v>
       </c>
-      <c r="C14" s="46">
+      <c r="C14" s="48">
         <v>45982</v>
       </c>
       <c r="D14" s="16">
         <v>1</v>
       </c>
-      <c r="E14" s="55" t="s">
+      <c r="E14" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7368,16 +7392,16 @@
       <c r="A15" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="46">
+      <c r="B15" s="48">
         <v>45980</v>
       </c>
-      <c r="C15" s="46">
+      <c r="C15" s="48">
         <v>45982</v>
       </c>
       <c r="D15" s="16">
         <v>1</v>
       </c>
-      <c r="E15" s="55" t="s">
+      <c r="E15" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7385,16 +7409,16 @@
       <c r="A16" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="46">
+      <c r="B16" s="48">
         <v>45980</v>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="48">
         <v>45982</v>
       </c>
       <c r="D16" s="16">
         <v>1</v>
       </c>
-      <c r="E16" s="55" t="s">
+      <c r="E16" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7402,16 +7426,16 @@
       <c r="A17" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="46">
+      <c r="B17" s="48">
         <v>45980</v>
       </c>
-      <c r="C17" s="46">
+      <c r="C17" s="48">
         <v>45982</v>
       </c>
       <c r="D17" s="16">
         <v>1</v>
       </c>
-      <c r="E17" s="55" t="s">
+      <c r="E17" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7419,16 +7443,16 @@
       <c r="A18" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="46">
+      <c r="B18" s="48">
         <v>45981</v>
       </c>
-      <c r="C18" s="46">
+      <c r="C18" s="48">
         <v>45983</v>
       </c>
       <c r="D18" s="16">
         <v>1</v>
       </c>
-      <c r="E18" s="55" t="s">
+      <c r="E18" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7436,16 +7460,16 @@
       <c r="A19" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="46">
+      <c r="B19" s="48">
         <v>45982</v>
       </c>
-      <c r="C19" s="46">
+      <c r="C19" s="48">
         <v>45984</v>
       </c>
       <c r="D19" s="16">
         <v>1</v>
       </c>
-      <c r="E19" s="55" t="s">
+      <c r="E19" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7453,16 +7477,16 @@
       <c r="A20" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="46">
+      <c r="B20" s="48">
         <v>45983</v>
       </c>
-      <c r="C20" s="46">
+      <c r="C20" s="48">
         <v>45985</v>
       </c>
       <c r="D20" s="16">
         <v>1</v>
       </c>
-      <c r="E20" s="55" t="s">
+      <c r="E20" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7470,16 +7494,16 @@
       <c r="A21" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="46">
+      <c r="B21" s="48">
         <v>45986</v>
       </c>
-      <c r="C21" s="46">
+      <c r="C21" s="48">
         <v>45987</v>
       </c>
       <c r="D21" s="16">
         <v>1</v>
       </c>
-      <c r="E21" s="55" t="s">
+      <c r="E21" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7487,16 +7511,16 @@
       <c r="A22" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="46">
+      <c r="B22" s="48">
         <v>45986</v>
       </c>
-      <c r="C22" s="46">
+      <c r="C22" s="48">
         <v>45987</v>
       </c>
       <c r="D22" s="16">
         <v>1</v>
       </c>
-      <c r="E22" s="55" t="s">
+      <c r="E22" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7504,16 +7528,16 @@
       <c r="A23" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="46">
+      <c r="B23" s="48">
         <v>45986</v>
       </c>
-      <c r="C23" s="46">
+      <c r="C23" s="48">
         <v>45987</v>
       </c>
       <c r="D23" s="16">
         <v>1</v>
       </c>
-      <c r="E23" s="55" t="s">
+      <c r="E23" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7521,16 +7545,16 @@
       <c r="A24" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="46">
+      <c r="B24" s="48">
         <v>45986</v>
       </c>
-      <c r="C24" s="46">
+      <c r="C24" s="48">
         <v>45987</v>
       </c>
       <c r="D24" s="16">
         <v>1</v>
       </c>
-      <c r="E24" s="55" t="s">
+      <c r="E24" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7538,16 +7562,16 @@
       <c r="A25" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="46">
+      <c r="B25" s="48">
         <v>45986</v>
       </c>
-      <c r="C25" s="46">
+      <c r="C25" s="48">
         <v>45987</v>
       </c>
       <c r="D25" s="16">
         <v>1</v>
       </c>
-      <c r="E25" s="55" t="s">
+      <c r="E25" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7555,16 +7579,16 @@
       <c r="A26" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="46">
+      <c r="B26" s="48">
         <v>45986</v>
       </c>
-      <c r="C26" s="46">
+      <c r="C26" s="48">
         <v>45987</v>
       </c>
       <c r="D26" s="16">
         <v>1</v>
       </c>
-      <c r="E26" s="55" t="s">
+      <c r="E26" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7572,16 +7596,16 @@
       <c r="A27" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="46">
+      <c r="B27" s="48">
         <v>45986</v>
       </c>
-      <c r="C27" s="46">
+      <c r="C27" s="48">
         <v>45987</v>
       </c>
       <c r="D27" s="16">
         <v>1</v>
       </c>
-      <c r="E27" s="55" t="s">
+      <c r="E27" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7589,16 +7613,16 @@
       <c r="A28" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="46">
+      <c r="B28" s="48">
         <v>45986</v>
       </c>
-      <c r="C28" s="46">
+      <c r="C28" s="48">
         <v>45987</v>
       </c>
       <c r="D28" s="16">
         <v>1</v>
       </c>
-      <c r="E28" s="55" t="s">
+      <c r="E28" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7606,16 +7630,16 @@
       <c r="A29" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="46">
+      <c r="B29" s="48">
         <v>45986</v>
       </c>
-      <c r="C29" s="46">
+      <c r="C29" s="48">
         <v>45987</v>
       </c>
       <c r="D29" s="16">
         <v>1</v>
       </c>
-      <c r="E29" s="55" t="s">
+      <c r="E29" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7623,16 +7647,16 @@
       <c r="A30" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B30" s="46">
+      <c r="B30" s="48">
         <v>45986</v>
       </c>
-      <c r="C30" s="46">
+      <c r="C30" s="48">
         <v>45987</v>
       </c>
       <c r="D30" s="16">
         <v>1</v>
       </c>
-      <c r="E30" s="55" t="s">
+      <c r="E30" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7640,16 +7664,16 @@
       <c r="A31" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="46">
+      <c r="B31" s="48">
         <v>45992</v>
       </c>
-      <c r="C31" s="46">
+      <c r="C31" s="48">
         <v>45993</v>
       </c>
       <c r="D31" s="16">
         <v>1</v>
       </c>
-      <c r="E31" s="55" t="s">
+      <c r="E31" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7657,16 +7681,16 @@
       <c r="A32" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="46">
+      <c r="B32" s="48">
         <v>45992</v>
       </c>
-      <c r="C32" s="46">
+      <c r="C32" s="48">
         <v>45993</v>
       </c>
       <c r="D32" s="16">
         <v>1</v>
       </c>
-      <c r="E32" s="55" t="s">
+      <c r="E32" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7674,16 +7698,16 @@
       <c r="A33" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="46">
+      <c r="B33" s="48">
         <v>45992</v>
       </c>
-      <c r="C33" s="46">
+      <c r="C33" s="48">
         <v>45993</v>
       </c>
       <c r="D33" s="16">
         <v>1</v>
       </c>
-      <c r="E33" s="55" t="s">
+      <c r="E33" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7691,16 +7715,16 @@
       <c r="A34" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="46">
+      <c r="B34" s="48">
         <v>45993</v>
       </c>
-      <c r="C34" s="46">
+      <c r="C34" s="48">
         <v>45993</v>
       </c>
       <c r="D34" s="16">
         <v>1</v>
       </c>
-      <c r="E34" s="55" t="s">
+      <c r="E34" s="57" t="s">
         <v>35</v>
       </c>
     </row>
@@ -8314,21 +8338,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="41" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="2" ht="409.5" spans="1:3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="43" t="s">
         <v>64</v>
       </c>
       <c r="C2" s="23" t="s">
@@ -8441,7 +8465,7 @@
       <c r="A15" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="44" t="s">
         <v>88</v>
       </c>
       <c r="C15" s="20"/>
@@ -8679,7 +8703,7 @@
       <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="34">
+      <c r="A2" s="36">
         <v>45962</v>
       </c>
       <c r="B2" s="20"/>
@@ -8688,7 +8712,7 @@
       <c r="A3" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="37" t="s">
         <v>91</v>
       </c>
     </row>
@@ -8696,7 +8720,7 @@
       <c r="A4" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="37" t="s">
         <v>93</v>
       </c>
     </row>
@@ -8704,21 +8728,21 @@
       <c r="A5" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="37" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="36">
+      <c r="A6" s="38">
         <v>45969</v>
       </c>
       <c r="B6" s="20"/>
     </row>
-    <row r="7" s="33" customFormat="1" ht="57.6" spans="1:2">
-      <c r="A7" s="37" t="s">
+    <row r="7" s="35" customFormat="1" ht="57.6" spans="1:2">
+      <c r="A7" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="40" t="s">
         <v>97</v>
       </c>
     </row>
@@ -8736,7 +8760,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="38.4444444444444" style="20" customWidth="1"/>
@@ -9526,6 +9550,14 @@
       </c>
       <c r="B87" s="18" t="s">
         <v>292</v>
+      </c>
+    </row>
+    <row r="88" ht="216" spans="1:2">
+      <c r="A88" s="33" t="s">
+        <v>293</v>
+      </c>
+      <c r="B88" s="34" t="s">
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -9595,7 +9627,7 @@
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="16" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" spans="1:1">
@@ -9633,7 +9665,7 @@
         <v>38</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="18" spans="1:1">
@@ -9643,76 +9675,76 @@
     </row>
     <row r="19" ht="72" spans="1:1">
       <c r="A19" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="20" ht="72" spans="1:1">
       <c r="A20" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="21" ht="100.8" spans="1:2">
       <c r="A21" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B22" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="23" ht="57.6" spans="1:2">
       <c r="A23" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="24" ht="72" spans="1:2">
       <c r="A24" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="25" ht="86.4" spans="1:2">
       <c r="A25" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="26" ht="43.2" spans="1:2">
       <c r="A26" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="27" ht="28.8" spans="1:2">
       <c r="A27" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="28" ht="43.2" spans="1:2">
       <c r="A28" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -9732,27 +9764,27 @@
   <sheetData>
     <row r="2" spans="1:1">
       <c r="A2" s="14" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="8" ht="15" spans="1:1">
       <c r="A8" s="15" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="9" ht="120" customHeight="1" spans="1:1">
       <c r="A9" s="9" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -9776,201 +9808,201 @@
   <sheetData>
     <row r="1" spans="2:3">
       <c r="B1" s="7" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2" spans="2:3">
       <c r="B2" s="8" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="8" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>323</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="8" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="8" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="8" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="8" ht="43.2" spans="2:3">
       <c r="B8" s="8" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="9" spans="2:2">
       <c r="B9" s="10" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="10" spans="2:2">
       <c r="B10" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="11" ht="23.4" spans="2:2">
       <c r="B11" s="11" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="12" spans="2:2">
       <c r="B12" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" spans="2:2">
       <c r="B13" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="14" spans="2:2">
       <c r="B14" s="12" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="15" spans="2:2">
       <c r="B15" s="12" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="16" spans="2:2">
       <c r="B16" s="12" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="17" spans="2:2">
       <c r="B17" s="12" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="18" spans="2:2">
       <c r="B18" s="12" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="19" spans="2:2">
       <c r="B19" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="20" spans="2:2">
       <c r="B20" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="21" spans="2:2">
       <c r="B21" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="22" spans="2:2">
       <c r="B22" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="23" spans="2:2">
       <c r="B23" s="12" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="24" spans="2:2">
       <c r="B24" s="12" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="25" spans="2:2">
       <c r="B25" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="26" ht="23.4" spans="2:2">
       <c r="B26" s="11" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="27" spans="2:2">
       <c r="B27" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="28" spans="2:2">
       <c r="B28" s="12" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="29" spans="2:2">
       <c r="B29" s="12" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="30" spans="2:2">
       <c r="B30" s="12" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="31" spans="2:2">
       <c r="B31" s="12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="32" spans="2:2">
       <c r="B32" s="12" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="33" spans="2:2">
       <c r="B33" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="34" spans="2:2">
       <c r="B34" s="12" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="35" spans="2:2">
       <c r="B35" s="12" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="36" spans="2:2">
@@ -9995,83 +10027,83 @@
     </row>
     <row r="40" spans="2:2">
       <c r="B40" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="41" ht="23.4" spans="2:2">
       <c r="B41" s="11" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="42" spans="2:2">
       <c r="B42" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="43" spans="2:2">
       <c r="B43" s="12" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="44" spans="2:2">
       <c r="B44" s="12" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="45" spans="2:2">
       <c r="B45" s="12" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="46" spans="2:2">
       <c r="B46" s="12" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="47" spans="2:2">
       <c r="B47" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="48" spans="2:2">
       <c r="B48" s="13" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="49" spans="2:2">
       <c r="B49" s="13" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="50" spans="2:2">
       <c r="B50" s="13" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="51" spans="2:2">
       <c r="B51" s="13" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="52" spans="2:2">
       <c r="B52" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="54" ht="13" customHeight="1"/>
     <row r="55" ht="22" customHeight="1" spans="2:2">
       <c r="B55" s="11" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="56" spans="2:2">
       <c r="B56" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="57" spans="2:2">
       <c r="B57" s="12" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="58" spans="2:2">
@@ -10086,17 +10118,17 @@
     </row>
     <row r="60" spans="2:2">
       <c r="B60" s="12" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="61" spans="2:2">
       <c r="B61" s="12" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="62" spans="2:2">
       <c r="B62" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
   </sheetData>
@@ -10113,7 +10145,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -10128,7 +10160,7 @@
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
       <c r="N1" s="5" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="O1" s="6"/>
       <c r="P1" s="6"/>
@@ -10370,7 +10402,7 @@
     </row>
     <row r="12" spans="1:21">
       <c r="A12" s="3" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -10556,7 +10588,7 @@
     </row>
     <row r="22" spans="1:21">
       <c r="A22" s="4" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>

</xml_diff>